<commit_message>
Update template file to push formatting to right one column
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/ProjectMap.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/ProjectMap.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19001"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brunworg\Source\Workspaces\genBOE\dev\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\Documents\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEC5F8B-1C77-4082-BD94-BFDF0131367E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="0" windowWidth="21570" windowHeight="7545"/>
+    <workbookView xWindow="270" yWindow="5070" windowWidth="38130" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PROJECTMAP" sheetId="1" r:id="rId1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Resources</t>
   </si>
@@ -106,19 +107,22 @@
     <t>Resource</t>
   </si>
   <si>
-    <t>Old Resource</t>
-  </si>
-  <si>
     <t>% Tier</t>
   </si>
   <si>
     <t>Legacy Resources</t>
+  </si>
+  <si>
+    <t>Business Resource Code</t>
+  </si>
+  <si>
+    <t>Legacy Resource</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -231,7 +235,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -508,32 +512,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:HQ1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:HR1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" style="9" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="9" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" style="9" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" style="9" customWidth="1"/>
-    <col min="5" max="7" width="13.140625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="6" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" style="10" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" style="9" customWidth="1"/>
-    <col min="13" max="13" width="22.28515625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" style="7" customWidth="1"/>
-    <col min="15" max="15" width="12.28515625" style="8" customWidth="1"/>
-    <col min="16" max="16" width="28.85546875" style="12" customWidth="1"/>
-    <col min="17" max="17" width="9.42578125" style="12" customWidth="1"/>
-    <col min="18" max="18" width="25.7109375" style="10" customWidth="1"/>
-    <col min="19" max="21" width="13.28515625" style="5" customWidth="1"/>
-    <col min="22" max="22" width="10.7109375" style="13" customWidth="1"/>
-    <col min="23" max="225" width="9.140625" style="12"/>
+    <col min="5" max="8" width="13.140625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" style="10" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="9" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="9" customWidth="1"/>
+    <col min="14" max="14" width="22.28515625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" style="8" customWidth="1"/>
+    <col min="17" max="17" width="28.85546875" style="12" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" style="12" customWidth="1"/>
+    <col min="19" max="19" width="25.7109375" style="10" customWidth="1"/>
+    <col min="20" max="22" width="13.28515625" style="5" customWidth="1"/>
+    <col min="23" max="23" width="10.7109375" style="13" customWidth="1"/>
+    <col min="24" max="226" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:225" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:226" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
@@ -553,54 +557,56 @@
         <v>18</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="W1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="W1" s="11"/>
       <c r="X1" s="11"/>
       <c r="Y1" s="11"/>
       <c r="Z1" s="11"/>
@@ -803,15 +809,20 @@
       <c r="HO1" s="11"/>
       <c r="HP1" s="11"/>
       <c r="HQ1" s="11"/>
+      <c r="HR1" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -839,7 +850,7 @@
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -855,5 +866,9 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>